<commit_message>
Replace with worksheet pipeline v1
Adds the full curriculum-aligned K-G3 unit generation pipeline: stage state
machine, schemas, drift gates (consistency, curriculum text, image-text
alignment), product-quality rubric publication gate, Slides deck builder,
clipart catalogue, Ontario MOE curriculum reference cache, and 5 generated
units across 3 batches (Pattern Parade K/G1/G2/G3 + Counting Crew K).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/canadian_classroom_content_batches.xlsx
+++ b/canadian_classroom_content_batches.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -121,8 +121,14 @@
       <color rgb="001C3B5A"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -162,6 +168,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EAD1DC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -235,7 +246,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -318,6 +329,20 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -980,7 +1005,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1116,10 +1141,18 @@
           <t>K now counts to 20 (was 10). Need activities beyond standard number lines. Manipulative-based.</t>
         </is>
       </c>
-      <c r="K4" s="24" t="inlineStr"/>
-      <c r="L4" s="25" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="K4" s="24" t="inlineStr">
+        <is>
+          <t>[2026-04-12 12:54] Generation failed: Unexpected error: "Could not resolve authentication method. Expected either api_key or auth_token to be set. Or for one of the `X-Api-Key` or `Authorization` headers to be explicitly omitted"
+[2026-04-12 12:58] Generation failed: API error: Connection error.
+[2026-04-12 13:18] Generation failed: API error: Connection error.
+[2026-04-12 13:38] Generation failed: Unexpected error: "Could not resolve authentication method. Expected either api_key or auth_token to be set. Or for one of the `X-Api-Key` or `Authorization` headers to be explicitly omitted"
+[2026-04-12 13:50] Generation failed: API error after 3 attempts: Connection error.</t>
+        </is>
+      </c>
+      <c r="L4" s="32" t="inlineStr">
+        <is>
+          <t>deprecated</t>
         </is>
       </c>
     </row>
@@ -1172,10 +1205,17 @@
           <t>Direct match to PDF example. Validates template quality vs. known benchmark.</t>
         </is>
       </c>
-      <c r="K5" s="24" t="inlineStr"/>
-      <c r="L5" s="25" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="K5" s="24" t="inlineStr">
+        <is>
+          <t>[2026-04-12 12:54] Generation failed: Unexpected error: "Could not resolve authentication method. Expected either api_key or auth_token to be set. Or for one of the `X-Api-Key` or `Authorization` headers to be explicitly omitted"
+[2026-04-12 13:01] Generation failed: API error: Connection error.
+[2026-04-12 13:21] Generation failed: API error: Connection error.
+[2026-04-12 14:04] Generation failed: API error after 3 attempts: Connection error.</t>
+        </is>
+      </c>
+      <c r="L5" s="32" t="inlineStr">
+        <is>
+          <t>deprecated</t>
         </is>
       </c>
     </row>
@@ -1228,10 +1268,16 @@
           <t>New 2023 curriculum. Almost no Ontario-specific morphology resources exist for Grade 2.</t>
         </is>
       </c>
-      <c r="K6" s="24" t="inlineStr"/>
-      <c r="L6" s="25" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="K6" s="24" t="inlineStr">
+        <is>
+          <t>[2026-04-12 12:54] Generation failed: Unexpected error: "Could not resolve authentication method. Expected either api_key or auth_token to be set. Or for one of the `X-Api-Key` or `Authorization` headers to be explicitly omitted"
+[2026-04-12 13:04] Generation failed: API error: Connection error.
+[2026-04-12 13:24] Generation failed: API error: Connection error.</t>
+        </is>
+      </c>
+      <c r="L6" s="32" t="inlineStr">
+        <is>
+          <t>deprecated</t>
         </is>
       </c>
     </row>
@@ -1284,10 +1330,17 @@
           <t>Coding is mandated but most resources require screens. Physical grid mats are the gap.</t>
         </is>
       </c>
-      <c r="K7" s="24" t="inlineStr"/>
-      <c r="L7" s="25" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="K7" s="24" t="inlineStr">
+        <is>
+          <t>[2026-04-12 12:54] Generation failed: Unexpected error: "Could not resolve authentication method. Expected either api_key or auth_token to be set. Or for one of the `X-Api-Key` or `Authorization` headers to be explicitly omitted"
+[2026-04-12 13:07] Generation failed: API error: Connection error.
+[2026-04-12 13:25] Generation failed: Unexpected error: "Could not resolve authentication method. Expected either api_key or auth_token to be set. Or for one of the `X-Api-Key` or `Authorization` headers to be explicitly omitted"
+[2026-04-12 13:27] Generation failed: API error: Connection error.</t>
+        </is>
+      </c>
+      <c r="L7" s="32" t="inlineStr">
+        <is>
+          <t>deprecated</t>
         </is>
       </c>
     </row>
@@ -1340,8 +1393,295 @@
           <t>SOR pivot. Decodable CVC focus. Tests Language strand output quality vs. Math strand.</t>
         </is>
       </c>
-      <c r="K8" s="24" t="inlineStr"/>
-      <c r="L8" s="25" t="inlineStr">
+      <c r="K8" s="24" t="inlineStr">
+        <is>
+          <t>[2026-04-12 12:54] Generation failed: Unexpected error: "Could not resolve authentication method. Expected either api_key or auth_token to be set. Or for one of the `X-Api-Key` or `Authorization` headers to be explicitly omitted"
+[2026-04-12 13:10] Generation failed: API error: Connection error.
+[2026-04-12 13:28] Generation failed: API error: Connection error.
+[2026-04-12 13:30] Generation failed: API error: Connection error.</t>
+        </is>
+      </c>
+      <c r="L8" s="32" t="inlineStr">
+        <is>
+          <t>deprecated</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Batch 1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Kindergarten</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>A. Patterns and Relationships</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Full Unit</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Pattern Parade</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>A7.1, A7.2, A7.3, A7.4</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>5</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Theme hook: Animals march in patterned lines through the classroom. Source: https://www.dcp.edu.gov.on.ca/en/curriculum/kindergarten/grades/jk-sk/a/a7</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>[2026-04-26 13:43] All 15 stages done. 35-page package: 5 lessons + 5 worksheets + 7 manipulatives + formative + reflection + 4 trackers + rubric + summative guide + certificate. $9.99 CAD suggested.</t>
+        </is>
+      </c>
+      <c r="L11" s="34" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Batch 1</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Kindergarten</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>A. Patterns and Relationships</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Full Unit</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Bead Bracelet Workshop</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>A7.1, A7.2, A7.3, A7.4</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>5</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Theme hook: Making, reading, and fixing beaded bracelets. Source: https://www.dcp.edu.gov.on.ca/en/curriculum/kindergarten/grades/jk-sk/a/a7</t>
+        </is>
+      </c>
+      <c r="L12" s="33" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Batch 1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Kindergarten</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>A. Patterns and Relationships</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Full Unit</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Patterns in the Forest</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>A7.1, A7.2, A7.3, A7.4</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>5</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Theme hook: Finding natural patterns: leaves, animal tracks, pinecones. Source: https://www.dcp.edu.gov.on.ca/en/curriculum/kindergarten/grades/jk-sk/a/a7</t>
+        </is>
+      </c>
+      <c r="L13" s="33" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Batch 1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Kindergarten</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>A. Patterns and Relationships</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Full Unit</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Mystery Pattern Detectives</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>A7.1, A7.2, A7.3, A7.4</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>5</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Theme hook: Solving missing-piece pattern puzzles. Source: https://www.dcp.edu.gov.on.ca/en/curriculum/kindergarten/grades/jk-sk/a/a7</t>
+        </is>
+      </c>
+      <c r="L14" s="33" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Batch 1</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Kindergarten</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>A. Patterns and Relationships</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Full Unit</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Sound and Movement Patterns</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>A7.1, A7.2, A7.3, A7.4</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>5</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Theme hook: Clap-stomp, tall-short, loud-quiet patterns. Source: https://www.dcp.edu.gov.on.ca/en/curriculum/kindergarten/grades/jk-sk/a/a7</t>
+        </is>
+      </c>
+      <c r="L15" s="33" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
@@ -1362,7 +1702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1480,26 +1820,14 @@
           <t>Step by Step: My First Coding Mat</t>
         </is>
       </c>
-      <c r="G4" s="27" t="inlineStr">
-        <is>
-          <t>C_K.1</t>
-        </is>
-      </c>
+      <c r="G4" s="27" t="n"/>
       <c r="H4" s="27" t="n">
-        <v>5</v>
-      </c>
-      <c r="I4" s="27" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J4" s="27" t="inlineStr">
-        <is>
-          <t>2026 mandate. No screen required. Arrow-based movement on physical grid.</t>
-        </is>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="I4" s="27" t="n"/>
+      <c r="J4" s="27" t="n"/>
       <c r="K4" s="27" t="inlineStr"/>
-      <c r="L4" s="25" t="inlineStr">
+      <c r="L4" s="35" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
@@ -1536,26 +1864,14 @@
           <t>Sound Safari: Sorting by Beginning Sounds</t>
         </is>
       </c>
-      <c r="G5" s="27" t="inlineStr">
-        <is>
-          <t>B_K.1</t>
-        </is>
-      </c>
+      <c r="G5" s="27" t="n"/>
       <c r="H5" s="27" t="n">
-        <v>5</v>
-      </c>
-      <c r="I5" s="27" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J5" s="27" t="inlineStr">
-        <is>
-          <t>Sound-first K resources. Play-centre style — sorting toys by initial phoneme.</t>
-        </is>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="I5" s="27" t="n"/>
+      <c r="J5" s="27" t="n"/>
       <c r="K5" s="27" t="inlineStr"/>
-      <c r="L5" s="25" t="inlineStr">
+      <c r="L5" s="35" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
@@ -1592,26 +1908,14 @@
           <t>Fair Shares: Fractions for Little Learners</t>
         </is>
       </c>
-      <c r="G6" s="27" t="inlineStr">
-        <is>
-          <t>B_K.3</t>
-        </is>
-      </c>
+      <c r="G6" s="27" t="n"/>
       <c r="H6" s="27" t="n">
-        <v>5</v>
-      </c>
-      <c r="I6" s="27" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J6" s="27" t="inlineStr">
-        <is>
-          <t>K now expected to understand equal sharing. Almost no K-level fraction resources exist.</t>
-        </is>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="I6" s="27" t="n"/>
+      <c r="J6" s="27" t="n"/>
       <c r="K6" s="27" t="inlineStr"/>
-      <c r="L6" s="25" t="inlineStr">
+      <c r="L6" s="35" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
@@ -2284,6 +2588,171 @@
       </c>
       <c r="K18" s="27" t="inlineStr"/>
       <c r="L18" s="25" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Batch 2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Grade 1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>C. Algebra (Patterns and Relationships)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Full Unit</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Pattern Parade</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>C1.1, C1.2, C1.3, C1.4</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>5</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>G1 expansion of K Pattern Parade. Reuses Coco + animals. Adds pattern rules, missing elements, whole numbers up to 50.</t>
+        </is>
+      </c>
+      <c r="L19" s="33" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Batch 2</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Grade 2</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>C. Algebra (Patterns and Relationships)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Full Unit</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Pattern Parade</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>C1.1, C1.2, C1.3, C1.4</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>5</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>G2 expansion. Adds growing/shrinking patterns, real-life contexts, tables of values, whole numbers up to 100.</t>
+        </is>
+      </c>
+      <c r="L20" s="33" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Batch 2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Grade 3</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>C. Algebra (Patterns and Relationships)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Full Unit</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Pattern Parade</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>C1.1, C1.2, C1.3, C1.4</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>5</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>G3 expansion. Adds operations in patterns, justification of predictions, shapes+numbers, whole numbers up to 1000.</t>
+        </is>
+      </c>
+      <c r="L21" s="33" t="inlineStr">
         <is>
           <t>pending</t>
         </is>

</xml_diff>